<commit_message>
Dia 17 - 10 de febrero de 2026
Hoy he seguido añadiendo indicadores.
Tras hablar con la doctora he resuelto todas las dudas que tenia ayer sobre ciertos indicadores.
Hemos redactado otro correo pidiendo ciertos datos que nos habíamos dejado la primera vez a ver si llegan en un tiempo razonable.
Estoy teniendo bastantes problemas con los ingresos por especialidad. Una vez calculado el indicador por cada unidad, algo que es muy sencillo y prácticamente directo con pandas, no soy capaz de mostrarlo en los gráficos correctamente.
Mañana seguiré intentándolo o lo que hare será realizar todos los indicadores y con el resto, a priori mas fáciles, terminados, finalizar este con mas tiempo.
</commit_message>
<xml_diff>
--- a/Datos/Datos_Necesitamos.xlsx
+++ b/Datos/Datos_Necesitamos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NICO\Desktop\Universidad\Practicas\Practicas-2026-Nicolas-Garcia-Gomez\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4937F688-A724-4D93-8F3E-7E257281B588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49B338A-1A11-439C-B917-89E1A670A51F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="75">
   <si>
     <t>Reingresos no programados en URCCPQ</t>
   </si>
@@ -183,15 +183,6 @@
       </rPr>
       <t>)</t>
     </r>
-  </si>
-  <si>
-    <t>Alta precoz o no planificada del servicio de medicina intensiva</t>
-  </si>
-  <si>
-    <t>(Num de enfermos con alta precoz o no planificada del SMI</t>
-  </si>
-  <si>
-    <t>Total de altas)</t>
   </si>
   <si>
     <t>Resucitacion precoz de la sepsis</t>
@@ -469,6 +460,27 @@
   <si>
     <t>Num total de días de TET) = vmi</t>
   </si>
+  <si>
+    <t>Problemas</t>
+  </si>
+  <si>
+    <t>Listado de verificacion</t>
+  </si>
+  <si>
+    <t>Cuagulopatia</t>
+  </si>
+  <si>
+    <t>Sedacion continuada vale con tener RASS o BIS</t>
+  </si>
+  <si>
+    <t>Cantidad de trasfusion</t>
+  </si>
+  <si>
+    <t>Resucitacion precoz = 3 parametros nuevos</t>
+  </si>
+  <si>
+    <t>Biogram al inicio y al final</t>
+  </si>
 </sst>
 </file>
 
@@ -497,7 +509,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -531,6 +543,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -571,7 +589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -616,6 +634,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -898,17 +922,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AB476"/>
+  <dimension ref="A1:AB475"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="68.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="118.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="106.21875" customWidth="1"/>
     <col min="4" max="4" width="50.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -921,7 +947,9 @@
         <v>3</v>
       </c>
       <c r="E1" s="6"/>
-      <c r="F1" s="1"/>
+      <c r="F1" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -946,7 +974,7 @@
       <c r="AB1" s="1"/>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="5" t="s">
@@ -961,7 +989,7 @@
       <c r="E2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="1"/>
+      <c r="F2" s="6"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
@@ -986,11 +1014,11 @@
       <c r="AB2" s="1"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="17" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>5</v>
@@ -1001,7 +1029,7 @@
       <c r="E3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F3" s="1"/>
+      <c r="F3" s="6"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -1026,7 +1054,7 @@
       <c r="AB3" s="1"/>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="9" t="s">
@@ -1041,7 +1069,7 @@
       <c r="E4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4" s="6"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -1066,11 +1094,11 @@
       <c r="AB4" s="1"/>
     </row>
     <row r="5" spans="1:28" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="17" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>5</v>
@@ -1081,7 +1109,7 @@
       <c r="E5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="1"/>
+      <c r="F5" s="8"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1106,7 +1134,7 @@
       <c r="AB5" s="1"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="17" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="9" t="s">
@@ -1121,7 +1149,7 @@
       <c r="E6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="1"/>
+      <c r="F6" s="6"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -1146,7 +1174,7 @@
       <c r="AB6" s="1"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="17" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="9" t="s">
@@ -1161,7 +1189,7 @@
       <c r="E7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="1"/>
+      <c r="F7" s="6"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -1189,20 +1217,22 @@
       <c r="A8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="9" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
+      <c r="F8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="16"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -1229,19 +1259,21 @@
       <c r="A9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="5" t="s">
         <v>27</v>
       </c>
       <c r="E9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="1"/>
+      <c r="F9" s="4" t="s">
+        <v>69</v>
+      </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -1269,19 +1301,21 @@
       <c r="A10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>29</v>
+      <c r="B10" s="9" t="s">
+        <v>62</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>30</v>
+      <c r="D10" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="1"/>
+      <c r="F10" s="4" t="s">
+        <v>74</v>
+      </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -1306,22 +1340,22 @@
       <c r="AB10" s="1"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>31</v>
+      <c r="A11" s="17" t="s">
+        <v>30</v>
       </c>
-      <c r="B11" s="9" t="s">
-        <v>65</v>
+      <c r="B11" s="5" t="s">
+        <v>57</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>32</v>
+      <c r="D11" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F11" s="1"/>
+      <c r="F11" s="6"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -1347,21 +1381,23 @@
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>60</v>
+      <c r="B12" s="10" t="s">
+        <v>63</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>69</v>
+      <c r="D12" s="6" t="s">
+        <v>32</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="1"/>
+      <c r="F12" s="4" t="s">
+        <v>70</v>
+      </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -1386,22 +1422,22 @@
       <c r="AB12" s="1"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>66</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" s="1"/>
+      <c r="F13" s="6"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -1429,19 +1465,21 @@
       <c r="A14" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>37</v>
+      <c r="B14" s="9" t="s">
+        <v>64</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
-      <c r="F14" s="1"/>
+      <c r="F14" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -1466,22 +1504,22 @@
       <c r="AB14" s="1"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>67</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="5" t="s">
         <v>40</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F15" s="1"/>
+      <c r="F15" s="6"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -1515,13 +1553,13 @@
       <c r="C16" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>43</v>
+      <c r="D16" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F16" s="1"/>
+      <c r="F16" s="6"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -1547,10 +1585,10 @@
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>5</v>
@@ -1561,7 +1599,7 @@
       <c r="E17" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F17" s="1"/>
+      <c r="F17" s="6"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1587,21 +1625,21 @@
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F18" s="1"/>
+      <c r="F18" s="6"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1627,21 +1665,21 @@
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>5</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="E19" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F19" s="1"/>
+      <c r="F19" s="6"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -1667,10 +1705,10 @@
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>48</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>5</v>
@@ -1681,7 +1719,9 @@
       <c r="E20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F20" s="1"/>
+      <c r="F20" s="4" t="s">
+        <v>72</v>
+      </c>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1709,19 +1749,19 @@
       <c r="A21" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>51</v>
+      <c r="B21" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>52</v>
+      <c r="D21" s="8" t="s">
+        <v>67</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
-      <c r="F21" s="1"/>
+      <c r="F21" s="6"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -1746,21 +1786,15 @@
       <c r="AB21" s="1"/>
     </row>
     <row r="22" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>53</v>
+      <c r="A22" s="11" t="s">
+        <v>51</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>63</v>
+      <c r="B22" s="12" t="s">
+        <v>54</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>6</v>
-      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
@@ -1786,11 +1820,11 @@
       <c r="AB22" s="1"/>
     </row>
     <row r="23" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A23" s="11" t="s">
-        <v>54</v>
+      <c r="A23" s="13" t="s">
+        <v>52</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -1820,12 +1854,10 @@
       <c r="AB23" s="1"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
-        <v>55</v>
+      <c r="A24" s="14" t="s">
+        <v>53</v>
       </c>
-      <c r="B24" s="12" t="s">
-        <v>58</v>
-      </c>
+      <c r="B24" s="15"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1854,10 +1886,8 @@
       <c r="AB24" s="1"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A25" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B25" s="15"/>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -9656,7 +9686,7 @@
       <c r="AB284" s="1"/>
     </row>
     <row r="285" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A285" s="2"/>
+      <c r="A285" s="3"/>
       <c r="B285" s="2"/>
       <c r="C285" s="2"/>
       <c r="D285" s="2"/>
@@ -9686,7 +9716,7 @@
       <c r="AB285" s="1"/>
     </row>
     <row r="286" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A286" s="3"/>
+      <c r="A286" s="1"/>
       <c r="B286" s="2"/>
       <c r="C286" s="2"/>
       <c r="D286" s="2"/>
@@ -10077,10 +10107,10 @@
     </row>
     <row r="299" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A299" s="1"/>
-      <c r="B299" s="2"/>
-      <c r="C299" s="2"/>
-      <c r="D299" s="2"/>
-      <c r="E299" s="2"/>
+      <c r="B299" s="1"/>
+      <c r="C299" s="1"/>
+      <c r="D299" s="1"/>
+      <c r="E299" s="1"/>
       <c r="F299" s="1"/>
       <c r="G299" s="1"/>
       <c r="H299" s="1"/>
@@ -15385,36 +15415,6 @@
       <c r="AA475" s="1"/>
       <c r="AB475" s="1"/>
     </row>
-    <row r="476" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A476" s="1"/>
-      <c r="B476" s="1"/>
-      <c r="C476" s="1"/>
-      <c r="D476" s="1"/>
-      <c r="E476" s="1"/>
-      <c r="F476" s="1"/>
-      <c r="G476" s="1"/>
-      <c r="H476" s="1"/>
-      <c r="I476" s="1"/>
-      <c r="J476" s="1"/>
-      <c r="K476" s="1"/>
-      <c r="L476" s="1"/>
-      <c r="M476" s="1"/>
-      <c r="N476" s="1"/>
-      <c r="O476" s="1"/>
-      <c r="P476" s="1"/>
-      <c r="Q476" s="1"/>
-      <c r="R476" s="1"/>
-      <c r="S476" s="1"/>
-      <c r="T476" s="1"/>
-      <c r="U476" s="1"/>
-      <c r="V476" s="1"/>
-      <c r="W476" s="1"/>
-      <c r="X476" s="1"/>
-      <c r="Y476" s="1"/>
-      <c r="Z476" s="1"/>
-      <c r="AA476" s="1"/>
-      <c r="AB476" s="1"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Dia 28 - 25 de febrero de 2026
Hoy he seguido intentando crear el archivo ejecutable pero ha ido a bastante peor.
Intentando solucionar los errores de ayer lo único que he conseguido ha sido hacer que ahora ni cargue la página por lo que tengo que hacer borrón y cuanta nueva porque no estoy yendo hacia buen camino.
Después he estado con la doctora recopilando los primeros datos y he modificado ciertos métodos.
Debido a nuevas necesidades de la doctora y que los datos artificiales que estaba utilizando no estaban correctos y habían desembocado en un calculo incorrecto.
</commit_message>
<xml_diff>
--- a/Datos/Datos_Necesitamos.xlsx
+++ b/Datos/Datos_Necesitamos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NICO\Desktop\Universidad\Practicas\Practicas-2026-Nicolas-Garcia-Gomez\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50DC183D-BE1D-4589-8B50-E3D32605535C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A164D693-29AB-4A99-92BC-6D425073A5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="69">
   <si>
     <t>Reingresos no programados en URCCPQ</t>
   </si>
@@ -460,6 +460,9 @@
   <si>
     <t>Num total de días de TET) = vmi</t>
   </si>
+  <si>
+    <t>ventana de sedacion es un numero</t>
+  </si>
 </sst>
 </file>
 
@@ -488,7 +491,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -522,6 +525,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -562,7 +571,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -610,6 +619,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1077,7 +1089,9 @@
       <c r="E5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="7"/>
+      <c r="F5" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1157,7 +1171,7 @@
       <c r="E7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="5"/>
+      <c r="F7" s="7"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>

</xml_diff>

<commit_message>
Dia 29 - 26 de febrero de 2026
Hoy he decidido volver a la solución que encontré el anterior día 26, a pesar de que se abría de forma infinita por lo menos, se abrían cosa que ayer no conseguí.
Esta ha sido en los primeros treinta minutos del día mientras esperaba a la doctora.
Después hemos empezado a pasar los datos de enero mas o menos llevaremos la mitad.
Mañana terminaremos todos los datos, podremos ver si los cálculos están correctos y si los datos recogidos son los idóneos.
</commit_message>
<xml_diff>
--- a/Datos/Datos_Necesitamos.xlsx
+++ b/Datos/Datos_Necesitamos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NICO\Desktop\Universidad\Practicas\Practicas-2026-Nicolas-Garcia-Gomez\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A164D693-29AB-4A99-92BC-6D425073A5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739DF0D0-B9D7-4531-972B-2E7612D55EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="68">
   <si>
     <t>Reingresos no programados en URCCPQ</t>
   </si>
@@ -460,9 +460,6 @@
   <si>
     <t>Num total de días de TET) = vmi</t>
   </si>
-  <si>
-    <t>ventana de sedacion es un numero</t>
-  </si>
 </sst>
 </file>
 
@@ -491,7 +488,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -525,12 +522,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -571,7 +562,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -619,9 +610,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1089,9 +1077,7 @@
       <c r="E5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="17" t="s">
-        <v>68</v>
-      </c>
+      <c r="F5" s="7"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>

</xml_diff>